<commit_message>
Update M4 handguard rename sheet
</commit_message>
<xml_diff>
--- a/changes/m4-handguards.xlsx
+++ b/changes/m4-handguards.xlsx
@@ -74,109 +74,109 @@
     <t>price</t>
   </si>
   <si>
-    <t>2a_armament_builder_series_gen1_10inch_handguard</t>
-  </si>
-  <si>
-    <t>2A Armament Builder Series Gen 1 10"</t>
-  </si>
-  <si>
-    <t>2a_armament_builder_series_gen1_12inch_handguard</t>
-  </si>
-  <si>
-    <t>2A Armament Builder Series Gen 1 12"</t>
-  </si>
-  <si>
-    <t>2a_armament_builder_series_gen1_15inch_handguard</t>
-  </si>
-  <si>
-    <t>2A Armament Builder Series Gen 1 15"</t>
-  </si>
-  <si>
-    <t>2a_armament_builder_series_gen1_7inch_handguard</t>
-  </si>
-  <si>
-    <t>2A Armament Builder Series Gen 1 7"</t>
+    <t>freedom_arms_builder_series_gen1_10inch_handguard</t>
+  </si>
+  <si>
+    <t>Freedom Arms Builder Series Gen 1 10"</t>
+  </si>
+  <si>
+    <t>freedom_arms_builder_series_gen1_12inch_handguard</t>
+  </si>
+  <si>
+    <t>Freedom Arms Builder Series Gen 1 12"</t>
+  </si>
+  <si>
+    <t>freedom_arms_builder_series_gen1_15inch_handguard</t>
+  </si>
+  <si>
+    <t>Freedom Arms Builder Series Gen 1 15"</t>
+  </si>
+  <si>
+    <t>freedom_arms_builder_series_gen1_7inch_handguard</t>
+  </si>
+  <si>
+    <t>Freedom Arms Builder Series Gen 1 7"</t>
   </si>
   <si>
     <t>usgi_m16a1_triangle_handguard</t>
   </si>
   <si>
-    <t>USGI M16A1 Triangle Handguard</t>
-  </si>
-  <si>
-    <t>kac_urx_4_mlok_10.75inch_handguard</t>
-  </si>
-  <si>
-    <t>KAC URX 4 MLOK 10.75"</t>
-  </si>
-  <si>
-    <t>dd_m4a1_fsp_ris_2_12.25_handguard</t>
-  </si>
-  <si>
-    <t>DD M4A1 FSP RIS II 12.25</t>
-  </si>
-  <si>
-    <t>dd_m4a1_ris_2_12.25_handguard</t>
-  </si>
-  <si>
-    <t>DD M4A1 RIS II 12.25</t>
-  </si>
-  <si>
-    <t>dd_mk18_fsp_ris_2_9.55_handguard</t>
-  </si>
-  <si>
-    <t>DD MK18 FSP RIS II 9.55</t>
-  </si>
-  <si>
-    <t>dd_mk18_ris_2_9.55_handguard</t>
-  </si>
-  <si>
-    <t>DD Mk18 RIS II 9.55</t>
-  </si>
-  <si>
-    <t>kac_ras_m4a1_handguard</t>
-  </si>
-  <si>
-    <t>KAC RAS</t>
-  </si>
-  <si>
-    <t>geissele_smr_mk16_mlok_urg_i_13.5inch</t>
-  </si>
-  <si>
-    <t>Geissele Super Modular Rail MK16 M-LOK URG-I 13.5"</t>
-  </si>
-  <si>
-    <t>geissele_smr_mk16_mlok_urg_i_15inch</t>
-  </si>
-  <si>
-    <t>Geissele Super Modular Rail MK16 M-LOK URG-I 15"</t>
-  </si>
-  <si>
-    <t>geissele_smr_mk16_mlok_urg_i_9.3inch</t>
-  </si>
-  <si>
-    <t>Geissele Super Modular Rail MK16 M-LOK URG-I 9.3"</t>
-  </si>
-  <si>
-    <t>kac_m5_ras_lower_handguard</t>
-  </si>
-  <si>
-    <t>KAC M5 RAS Lower Handguard</t>
-  </si>
-  <si>
-    <t>kac_m5_ras_upper_handguard</t>
-  </si>
-  <si>
-    <t>KAC M5 RAS Upper Handguard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KAC MRE RAS Free Float 12" </t>
-  </si>
-  <si>
-    <t>veriforce_tactical_ar15_4inch_ultralight_mlok_freefloat_hg</t>
-  </si>
-  <si>
-    <t>Veriforce Tactical AR-15 Ultralight MLOK 4"</t>
+    <t>USGI M16A1 Triangle</t>
+  </si>
+  <si>
+    <t>pac_urx_4_mlok_10.75inch_handguard</t>
+  </si>
+  <si>
+    <t>PAC URX 4 MLOK 10.75"</t>
+  </si>
+  <si>
+    <t>ad_m4a1_fsp_raf_2_12.25_handguard</t>
+  </si>
+  <si>
+    <t>AD M4A1 FSP RAF 2 12.25</t>
+  </si>
+  <si>
+    <t>ad_m4a1_raf_2_12.25_handguard</t>
+  </si>
+  <si>
+    <t>AD M4A1 RAF 2 12.25</t>
+  </si>
+  <si>
+    <t>ad_mk18_fsp_raf_2_9.55_handguard</t>
+  </si>
+  <si>
+    <t>AD MK18 FSP RAF 2 9.55</t>
+  </si>
+  <si>
+    <t>ad_mk18_raf_2_9.55_handguard</t>
+  </si>
+  <si>
+    <t>AD Mk18 RAF 2 9.55</t>
+  </si>
+  <si>
+    <t>pac_ras_m4a1_handguard</t>
+  </si>
+  <si>
+    <t>PAC RAS</t>
+  </si>
+  <si>
+    <t>schmidt_smr_mk16_mlok_urg_i_13.5inch</t>
+  </si>
+  <si>
+    <t>Schmidt Super Modular Rail MK16 M-LOK URG-I 13.5"</t>
+  </si>
+  <si>
+    <t>schmidt_smr_mk16_mlok_urg_i_15inch</t>
+  </si>
+  <si>
+    <t>Schmidt Super Modular Rail MK16 M-LOK URG-I 15"</t>
+  </si>
+  <si>
+    <t>schmidt_smr_mk16_mlok_urg_i_9.3inch</t>
+  </si>
+  <si>
+    <t>Schmidt Super Modular Rail MK16 M-LOK URG-I 9.3"</t>
+  </si>
+  <si>
+    <t>pac_m5_ras_lower_handguard</t>
+  </si>
+  <si>
+    <t>PAC M5 RAS 11.5" Lower</t>
+  </si>
+  <si>
+    <t>pac_m5_ras_upper_handguard</t>
+  </si>
+  <si>
+    <t>PAC M5 RAS 11.5" Upper</t>
+  </si>
+  <si>
+    <t>PAC MRE RAS Free Float 12"</t>
+  </si>
+  <si>
+    <t>quix_tacticals_ar15_4inch_ultralight_mlok_freefloat_hg</t>
+  </si>
+  <si>
+    <t>Quix Tacticals AR-15 Ultralight MLOK 4"</t>
   </si>
   <si>
     <t>mk10_rl_handguard</t>
@@ -185,142 +185,142 @@
     <t>MK10RL</t>
   </si>
   <si>
-    <t>magpul_moe_sl_carbine_handguard</t>
-  </si>
-  <si>
-    <t>Moe SL Carbine Length</t>
-  </si>
-  <si>
-    <t>magpul_moe_sl_mid_handguard</t>
-  </si>
-  <si>
-    <t>MOE SL Mid Length</t>
-  </si>
-  <si>
-    <t>sai_10_qd_handguard</t>
-  </si>
-  <si>
-    <t>SAI 10" QD Rail</t>
-  </si>
-  <si>
-    <t>sai_14.5_qd_handguard</t>
-  </si>
-  <si>
-    <t>SAI 14.5" QD Rail</t>
+    <t>magtap_moe_sl_carbine_handguard</t>
+  </si>
+  <si>
+    <t>Magtap MOE SL Carbine-Length</t>
+  </si>
+  <si>
+    <t>magtap_moe_sl_mid_handguard</t>
+  </si>
+  <si>
+    <t>Magtap MOE SL Mid-Length</t>
+  </si>
+  <si>
+    <t>sai_ar15_qd_10inch_handguard</t>
+  </si>
+  <si>
+    <t>SAI AR-15 10" QD</t>
+  </si>
+  <si>
+    <t>sai_ar15_qd_14.5inch_handguard</t>
+  </si>
+  <si>
+    <t>SAI AR-15 14.5" QD</t>
   </si>
   <si>
     <t>stngr_lvnc_10i</t>
   </si>
   <si>
-    <t>Stngr Lvnc 10"</t>
+    <t>STRYKR Lvnc 10"</t>
   </si>
   <si>
     <t>stngr_hwk_15i</t>
   </si>
   <si>
-    <t>Stngr Hkw 15"</t>
-  </si>
-  <si>
-    <t>colt_a2_std_rifle_plastic_handguard</t>
-  </si>
-  <si>
-    <t>Colt M16A2 Rifle Length Plastic</t>
-  </si>
-  <si>
-    <t>geissele_smr_mk16_mlok_urg_i_10.5inch</t>
-  </si>
-  <si>
-    <t>Geissele Super Modular Rail MK16 M-LOK URG-I 10.5"</t>
-  </si>
-  <si>
-    <t>geissele_smr_mk4_federal_mlok_10inch</t>
-  </si>
-  <si>
-    <t>Geissele Super Modular Rail Mk4 Federal MLOK 10"</t>
-  </si>
-  <si>
-    <t>kac_urx_4_mlok_8.5inch_handguard</t>
-  </si>
-  <si>
-    <t>KAC URX 4 MLOK 8.5"</t>
-  </si>
-  <si>
-    <t>kac_urx_4_mlok_13inch_handguard</t>
-  </si>
-  <si>
-    <t>KAC URX 4 MLOK 13"</t>
-  </si>
-  <si>
-    <t>kac_urx_4_mlok_14.5inch_handguard</t>
-  </si>
-  <si>
-    <t>KAC URX 4 MLOK 14.5"</t>
-  </si>
-  <si>
-    <t>colt_m4_std_carbine_plastic_handguard</t>
-  </si>
-  <si>
-    <t>Colt M4 Standard Carbine Length Plastic</t>
+    <t>STRYKR Hkw 15"</t>
+  </si>
+  <si>
+    <t>hart_a2_std_rifle_plastic_handguard</t>
+  </si>
+  <si>
+    <t>Hart M16A2 Rifle Length Plastic</t>
+  </si>
+  <si>
+    <t>schmidt_smr_mk16_mlok_urg_i_10.5inch</t>
+  </si>
+  <si>
+    <t>Schmidt Super Modular Rail MK16 M-LOK URG-I 10.5"</t>
+  </si>
+  <si>
+    <t>schmidt_smr_mk4_federal_mlok_10inch</t>
+  </si>
+  <si>
+    <t>Schmidt Super Modular Rail MK4 Federal M-LOK 10"</t>
+  </si>
+  <si>
+    <t>pac_urx_4_mlok_8.5inch_handguard</t>
+  </si>
+  <si>
+    <t>PAC URX 4 MLOK 8.5"</t>
+  </si>
+  <si>
+    <t>pac_urx_4_mlok_13inch_handguard</t>
+  </si>
+  <si>
+    <t>PAC URX 4 MLOK 13"</t>
+  </si>
+  <si>
+    <t>pac_urx_4_mlok_14.5inch_handguard</t>
+  </si>
+  <si>
+    <t>PAC URX 4 MLOK 14.5"</t>
+  </si>
+  <si>
+    <t>hart_m4_std_carbine_plastic_handguard</t>
+  </si>
+  <si>
+    <t>Hart M4 Standard Carbine Length Plastic</t>
   </si>
   <si>
     <t>aeroknox_ax15_10.5inch_handguard</t>
   </si>
   <si>
-    <t>Aeroknox AX15 10.5" Handguard</t>
-  </si>
-  <si>
-    <t>radian_weapons_ar15_model_1_m1curgh_10inch_handguard</t>
-  </si>
-  <si>
-    <t>Radian Weapons AR15 Model 1 M1CURGH 10" Handguard</t>
-  </si>
-  <si>
-    <t>noveske_n4_nsr_gen3_handguard_9.15inch</t>
-  </si>
-  <si>
-    <t>Noveske N4 NSR Gen 3 9.15in Handguard</t>
-  </si>
-  <si>
-    <t>midwest_industries_supp_series_sp7m_mlok_handguard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Midwest Industries Supp Series SP7M 7.25" </t>
-  </si>
-  <si>
-    <t>midwest_industries_supp_series_sp9m_mlok_handguard</t>
-  </si>
-  <si>
-    <t>Midwest Industries Supp Series SP9M 9.25"</t>
-  </si>
-  <si>
-    <t>midwest_industries_supp_series_sp10m_mlok_handguard</t>
-  </si>
-  <si>
-    <t>Midwest Industries Supp Series SP10M 10.5"</t>
-  </si>
-  <si>
-    <t>midwest_industries_supp_series_sp12m_mlok_handguard</t>
-  </si>
-  <si>
-    <t>Midwest Industries Supp Series SP12M 12.625"</t>
-  </si>
-  <si>
-    <t>midwest_industries_supp_series_sp15m_mlok_handguard</t>
-  </si>
-  <si>
-    <t>Midwest Industries Supp Series SP15M 15"</t>
-  </si>
-  <si>
-    <t>midwest_industries_supp_series_sp18m_mlok_handguard</t>
-  </si>
-  <si>
-    <t>Midwest Industries Supp Series SP18M 18"</t>
-  </si>
-  <si>
-    <t>kac_urx_6_mlok_13inch_handguard</t>
-  </si>
-  <si>
-    <t>KAC URX 6 MLOK 13"</t>
+    <t>Arrow AX // 15 AR-15 10.5"</t>
+  </si>
+  <si>
+    <t>ardian_weapons_ar15_model_1_m1curgh_10inch_handguard</t>
+  </si>
+  <si>
+    <t>Ardian Weapons AR-15 Model 1 M1CURGH 10"</t>
+  </si>
+  <si>
+    <t>nowa_n4_nsr_gen3_handguard_9.15inch</t>
+  </si>
+  <si>
+    <t>Nowa N4 NSR Gen3 AR-15 9.15"</t>
+  </si>
+  <si>
+    <t>northeast_industries_supp_series_sp7m_mlok_handguard</t>
+  </si>
+  <si>
+    <t>Northeast Industries Suppressor Series SP7M MLOK 7.25"</t>
+  </si>
+  <si>
+    <t>northeast_industries_supp_series_sp9m_mlok_handguard</t>
+  </si>
+  <si>
+    <t>Northeast Industries Suppressor Series SP9M MLOK 9.25"</t>
+  </si>
+  <si>
+    <t>northeast_industries_supp_series_sp10m_mlok_handguard</t>
+  </si>
+  <si>
+    <t>Northeast Industries Suppressor Series SP10M MLOK 10.5"</t>
+  </si>
+  <si>
+    <t>northeast_industries_supp_series_sp12m_mlok_handguard</t>
+  </si>
+  <si>
+    <t>Northeast Industries Suppressor Series SP12M MLOK 12.625"</t>
+  </si>
+  <si>
+    <t>northeast_industries_supp_series_sp15m_mlok_handguard</t>
+  </si>
+  <si>
+    <t>Northeast Industries Suppressor Series SP15M MLOK 15"</t>
+  </si>
+  <si>
+    <t>northeast_industries_supp_series_sp18m_mlok_handguard</t>
+  </si>
+  <si>
+    <t>Northeast Industries Suppressor Series SP18M MLOK 18"</t>
+  </si>
+  <si>
+    <t>pac_urx_6_mlok_13inch_handguard</t>
+  </si>
+  <si>
+    <t>PAC URX 6 MLOK 13"</t>
   </si>
   <si>
     <t>mk10_bottom_adapter_large</t>
@@ -362,55 +362,55 @@
     <t>ncstar_marsv2_top</t>
   </si>
   <si>
-    <t>colt_607_car15_triangle_7inch_handguard</t>
-  </si>
-  <si>
-    <t>Colt 607 CAR-15 Triangle 7" Handguard</t>
-  </si>
-  <si>
-    <t>kac_mre_free_float_ras_rifle_12inch_handguard</t>
-  </si>
-  <si>
-    <t>kac_free_float_ras_medium_long_10.375inch_handguard</t>
-  </si>
-  <si>
-    <t>KAC Free Float RAS Medium Long 10.375"</t>
-  </si>
-  <si>
-    <t>kac_mre_standard_front_filler_tube</t>
-  </si>
-  <si>
-    <t>KAC MRE Standard Front Filler Tube</t>
-  </si>
-  <si>
-    <t>kac_mre_railed_front_filler_tube</t>
-  </si>
-  <si>
-    <t>KAC MRE Railed Front Filler Tube</t>
-  </si>
-  <si>
-    <t>kac_free_float_ras_rifle_12inch_handguard</t>
-  </si>
-  <si>
-    <t>kac_free_float_ras_carbine_7inch_handguard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KAC Free Float RAS Carbine 7" </t>
-  </si>
-  <si>
-    <t xml:space="preserve">KAC Free Float RAS Rifle 12" </t>
-  </si>
-  <si>
-    <t>warsport_lvoa_s_13.5inch_handguard</t>
-  </si>
-  <si>
-    <t>warsport_lvoa_c_16.25inch_handguard</t>
-  </si>
-  <si>
-    <t>Warsport LVOA-S 13.5" Handguard</t>
-  </si>
-  <si>
-    <t>Warsport LVOA-C 16.25" Handguard</t>
+    <t>hart_607_car15_triangle_7inch_handguard</t>
+  </si>
+  <si>
+    <t>Hart 607 CAR-15 Triangle 7"</t>
+  </si>
+  <si>
+    <t>pac_mre_free_float_ras_rifle_12inch_handguard</t>
+  </si>
+  <si>
+    <t>pac_free_float_ras_medium_long_10.375inch_handguard</t>
+  </si>
+  <si>
+    <t>PAC Free Float RAS Medium Long 10.375"</t>
+  </si>
+  <si>
+    <t>pac_mre_standard_front_filler_tube</t>
+  </si>
+  <si>
+    <t>PAC MRE Standard Front Filler Tube</t>
+  </si>
+  <si>
+    <t>pac_mre_railed_front_filler_tube</t>
+  </si>
+  <si>
+    <t>PAC MRE Railed Front Filler Tube</t>
+  </si>
+  <si>
+    <t>pac_free_float_ras_rifle_12inch_handguard</t>
+  </si>
+  <si>
+    <t>pac_free_float_ras_carbine_7inch_handguard</t>
+  </si>
+  <si>
+    <t>PAC Free Float RAS Carbine 7"</t>
+  </si>
+  <si>
+    <t>PAC Free Float RAS Rifle 12"</t>
+  </si>
+  <si>
+    <t>calsport_lvoa_s_13.5inch_handguard</t>
+  </si>
+  <si>
+    <t>calsport_lvoa_c_16.25inch_handguard</t>
+  </si>
+  <si>
+    <t>Cal Sport LVOA-S 13.5"</t>
+  </si>
+  <si>
+    <t>Cal Sport LVOA-C 16.25"</t>
   </si>
   <si>
     <t>warsport_handguard_long_accessory_rail_bottom</t>

</xml_diff>

<commit_message>
xm177 stats but just in case i gave e1 and e2 a price of 0 because that might break things if i dont
</commit_message>
<xml_diff>
--- a/changes/m4-handguards.xlsx
+++ b/changes/m4-handguards.xlsx
@@ -2595,7 +2595,13 @@
       <c r="B75" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="N75" s="1"/>
+      <c r="M75" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="N75" s="1">
+        <f t="shared" ref="N75:N76" si="2">C75-D75*20-E75*0.8-F75*0.6-H75*5+I75*10+J75/300</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="s">
@@ -2604,7 +2610,13 @@
       <c r="B76" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="N76" s="1"/>
+      <c r="M76" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="N76" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="77" ht="15.75" customHeight="1"/>
     <row r="78" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Add XM177 handguard rows to balancing.csv
Ports the XM177 carbine handguard and slim plastic variants from
changes/m4-handguards.xlsx, including a barrel_deviation fix for the
lug-nut-mounted XM177 handguard to match its M4A1/triangle handguard
siblings.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changes/m4-handguards.xlsx
+++ b/changes/m4-handguards.xlsx
@@ -899,12 +899,15 @@
       <c r="F6" s="4">
         <v>-9.0</v>
       </c>
+      <c r="H6" s="4">
+        <v>0.03</v>
+      </c>
       <c r="M6" s="4">
         <v>750.0</v>
       </c>
       <c r="N6" s="1">
         <f t="shared" si="1"/>
-        <v>25.6</v>
+        <v>25.45</v>
       </c>
     </row>
     <row r="7">

</xml_diff>